<commit_message>
Incorporate user-provided Lexology text into Decreto 79/2017 recode
Align policy objective, instrument descriptions, and comments with Lexology
analysis. Add full Lexology text to English translation Word document.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Mozambique_4P_Index_Decreto_79_2017.xlsx
+++ b/Mozambique_4P_Index_Decreto_79_2017.xlsx
@@ -594,7 +594,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -667,7 +667,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Plastics relevance: Annex I typology includes all plastic types including polystyrene foam. Lexology/VdA analysis confirms hierarchy as core EPR design element.</t>
+          <t>Lexology: scope covers any packaging 'regardless of the materials used' plus collectable packaging waste. Annex I includes all plastic types including polystyrene foam.</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -699,7 +699,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I3" s="3" t="n">
@@ -780,7 +780,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -792,7 +792,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
@@ -833,7 +833,7 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Art. 5: Assigns competencies to Environment Ministry (rules, fiscalization, monitoring, valorisation oversight), Industry/Commerce Ministry (import/production standards), and Finance Ministry (tax/fine collection, customs clearance control).</t>
+          <t>Art. 5: Environment Ministry drafts/discloses rules, supervises and imposes sanctions; Industry and Commerce Ministry sets import/production standards; Finance Ministry collects fees and fines and supervises packaging rules at customs clearance (Lexology).</t>
         </is>
       </c>
       <c r="S4" s="3" t="n">
@@ -844,7 +844,7 @@
       </c>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>'Compete ao Ministério que superintende a área do Ambiente' fiscalizar, sancionar e monitorar; MIC define normas de produção/importação; MEF garante cobrança de taxas e controlo aduaneiro. Multi-ministry coordination (+0.25). Africa RISE/Imani project 2022–2025 supported TAE diploma and COMAGE operationalisation (+0.25).</t>
+          <t>Lexology confirms Art. 5 ministry competencies for Environment (rules, supervision, sanctions), Industry/Commerce (standards), Finance (fee/fine collection, customs). Multi-ministry coordination (+0.25). Africa RISE/Imani 2022–2025 supported TAE diploma and COMAGE operationalisation (+0.25).</t>
         </is>
       </c>
       <c r="V4" s="3">
@@ -853,7 +853,7 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>Multi-level governance (Rule 11); Decreto Art. 2 assigns MTA, MIC, MEF implementation.</t>
+          <t>Lexology: effectiveness depends on operation of entities in extended responsibility framework. Decreto Art. 2 assigns MTA, MIC, MEF implementation.</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -885,7 +885,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I5" s="3" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -978,7 +978,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I6" s="3" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Art. 7: Producers and importers co-responsible for packaging and packaging-waste management — must pay TAE fees and ensure return/valorisation of packaging waste directly or through recovery organisations.</t>
+          <t>Art. 7: Producers and importers jointly responsible for packaging and packaging-waste management; must pay packaging management fees; must ensure return and recovery of packaging waste directly or through recovery organisations (Lexology).</t>
         </is>
       </c>
       <c r="S6" s="3" t="n">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>'Os produtores e importadores são co-responsáveis pela gestão das embalagens e resíduos de embalagens.' Mandatory co-responsibility (+0.25). TAE payment obligation (+0.25) operationalising via DM 26/2025. Take-back/valorisation weakly implemented for plastics (IUCN 2022; VdA 2018 anticipates significant business impact).</t>
+          <t>Lexology: producers/importers 'jointly responsible' for management, fee payment, and return/recovery (+0.25 each obligation). TAE fee system operationalising via DM 26/2025 (+0.25). Lexology anticipates 'considerable impact on companies' — take-back/recovery weakly implemented for plastics (IUCN 2022).</t>
         </is>
       </c>
       <c r="V6" s="3">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>Core EPR obligation. Annex I explicitly covers all plastic types including polystyrene foam (item 1.2).</t>
+          <t>Core EPR obligation per Lexology. Scope includes all packaging materials; Annex I item 1.2 covers all plastic types including polystyrene foam.</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I7" s="3" t="n">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Art. 8: Waste operators must ensure environmentally safe, sustainable management favouring reduction, recycling and reuse; promote environmental education; and register with the Environment Ministry.</t>
+          <t>Art. 8: Waste operators must ensure environmentally safe, sustainable and rational packaging management (reduce, recycle, reuse; sorting, collection, handling, transport, storage and/or disposal); protect health and environment; promote community education; and register with Environment Ministry (Lexology).</t>
         </is>
       </c>
       <c r="S7" s="3" t="n">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>'Assegurar uma gestão ambientalmente segura, sustentável e racional das embalagens, tendo em conta a necessidade da sua redução, reciclagem e reutilização.' Registration requirement (+0.25). Limited evidence of comprehensive operator registration for plastic packaging streams.</t>
+          <t>Lexology lists four operator duties: safe management, health/environment protection, community education, Environment Ministry registration. Registration (+0.25). Limited evidence of comprehensive operator registration for plastic packaging streams.</t>
         </is>
       </c>
       <c r="V7" s="3">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="W7" s="2" t="inlineStr">
         <is>
-          <t>Applies to licensed operators handling plastic packaging waste.</t>
+          <t>Lexology attributes separate responsibilities to waste operators alongside producers.</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I8" s="3" t="n">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>'A responsabilidade do produtor e importador de embalagens é assumida através dos seguintes sistemas' (internal management, TAE, normalisation). Framework operative (+0.25). IUCN 2022 / Lexology-type analysis: only TAE system substantially implemented; internal management and normalisation need greater producer investment.</t>
+          <t>Lexology: producers/importers assume responsibility through Internal Management, Packaging Environmental Fee, and Packaging Standardisation systems. Framework operative (+0.25). Lexology observations: companies must manage waste through all three systems; effectiveness depends on complementary legislation and entity operation.</t>
         </is>
       </c>
       <c r="V8" s="3">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>Overarching EPR architecture instrument; one row for Art. 9 system design.</t>
+          <t>Overarching EPR architecture per Lexology. One row for Art. 9 system design.</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I9" s="3" t="n">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Art. 11: Direct internal management — producers/importers may individually or jointly pursue reduction, reuse, recycling, organic recovery, energy recovery or incineration; consumers pay a deposit at purchase refunded on return of used packaging.</t>
+          <t>Art. 11: Direct Internal Management System — producer/importer may opt individually or jointly for reduction, re-use, recycling, organic recovery, energetic recovery or incineration; consumer pays deposit at purchase reimbursed on return of used packaging (Lexology).</t>
         </is>
       </c>
       <c r="S9" s="3" t="n">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>'o consumidor de produtos que utilizem embalagens paga um determinado valor de depósito no acto da compra, que lhe é devolvido aquando da entrega da embalagem utilizada.' Deposit-return mechanism defined (+0.25). No national deposit system evidenced operational for plastic packaging (IUCN recommends Maputo pilot).</t>
+          <t>Lexology: deposit 'reimbursed once the used packaging is returned.' Mechanism defined (+0.25). Adopted at producer initiative — no national DRS evidenced operational for plastic packaging (IUCN recommends Maputo pilot).</t>
         </is>
       </c>
       <c r="V9" s="3">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>Deposit-return (DRS) for packaging including plastics. Art. 20(2)(a) penalises refusal to accept used packaging or refund deposits (15 minimum wages).</t>
+          <t>Lexology Internal Management System (direct form). Art. 20(2)(a): refusal to accept used packaging or refund deposit — 15 minimum wages.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I10" s="3" t="n">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>Art. 12: Indirect internal management — producers/importers may contract licensed waste operators (PRO-type entities) for collection, selective sorting, take-back and valorisation; financial counterparties required; responsibility transfers upon certified operator assumption declaration.</t>
+          <t>Art. 12: Indirect Internal Management System — producer/importer responsibility for packaging treatment transferred contractually to licensed entity; producer bears financial costs of selective collection, sorting, take-back and recovery; responsibility ends upon certified operator declaration of assumption (Lexology).</t>
         </is>
       </c>
       <c r="S10" s="3" t="n">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>'A responsabilidade dos produtores ou importadores... pode ser transferida, mediante celebração de contrato, para uma entidade devidamente licenciada.' PRO framework defined (+0.25). IUCN: indirect management system not yet operational at scale; producer inventories and PRO mandates need development.</t>
+          <t>Lexology: contractual transfer to licensed operator; producer bears collection/sorting/take-back/recovery costs (+0.25). Responsibility ends on operator assumption declaration (+0.25 framework). Not yet operational at scale (IUCN 2022).</t>
         </is>
       </c>
       <c r="V10" s="3">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>Mozambique PRO/contractual EPR model per VdA and IUCN analysis.</t>
+          <t>Lexology Indirect Internal Management System; PRO-type contractual EPR model.</t>
         </is>
       </c>
     </row>
@@ -1431,7 +1431,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Art. 13–14: Creates variable Packaging Environmental Fee (TAE) payable by all packaging producers and importers, based on environmental/public-health impact and treatment complexity; criteria include returnability, decomposition time/impact, treatment cost, and eco-design.</t>
+          <t>Art. 13: Packaging Environmental Fee (TAE / Taxa Ambiental sobre a Embalagem) payable by all packaging producers and importers; fee varies by environmental/public-health impact and waste-treatment complexity. AT charges imports; domestic producers pay annually on production report (Lexology).</t>
         </is>
       </c>
       <c r="S11" s="3" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="U11" s="2" t="inlineStr">
         <is>
-          <t>'É criada a Taxa Ambiental sobre a Embalagem (TAE).' DM 26/2025 (10 March 2025) defines formula, categories and exemptions per Art. 15 (+0.25). Levied on primary packaging including plastic (+0.25). AT collects on imports; annual production reports for domestic producers (Art. 16). Payment from 2026 after management-plan period (Club of Mozambique/Lusa). Up to 90% reduction when internal management established.</t>
+          <t>Lexology: TAE created Art. 13; AT collects imported packaging; annual production-report basis for domestic producers (+0.25 each). DM 26/2025 defines formula per Art. 15 (Lexology flagged need for complementary legislation) (+0.25). Levied on plastic packaging; payment from 2026; up to 90% reduction with internal management system.</t>
         </is>
       </c>
       <c r="V11" s="3">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>Previously scored in_force=0 pending diploma; DM 26/2025 operationalises Art. 15. Lexology URL and Africa RISE project document TAE as primary implemented EPR pillar.</t>
+          <t>Lexology Packaging Environmental Fee System. Complementary diploma DM 26/2025 (March 2025) addresses Lexology observation on regulatory legislation dependency.</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I12" s="3" t="n">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I13" s="3" t="n">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>Art. 17: Packaging normalisation — packaging must preferentially use biodegradable materials or materials permitting reuse, recycling or recovery; producers must limit volume/weight, design for returnability, and ensure recyclability. Applies to manufacturers, material suppliers, importers and distributors.</t>
+          <t>Art. 17: Packaging Standardisation System — packaging produced with preferably biodegradable or re-usable/recyclable/recoverable materials; producers, manufacturers, material suppliers and importers must ensure volume/weight limits, technical returnability, and recyclability (Lexology).</t>
         </is>
       </c>
       <c r="S13" s="3" t="n">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="U13" s="2" t="inlineStr">
         <is>
-          <t>'As embalagens devem ser produzidas com materiais preferencialmente de natureza biodegradável ou que permitam a reutilização, reciclagem ou valorização' and 'Recicláveis.' Mandatory language (+0.25). Art. 20(2)(d): market placement without packaging norms — 15 min. wages (+0.25). VdA notes significant business impact; limited enforcement data for plastic streams.</t>
+          <t>Lexology: three standardisation requirements — volume/dimension limits, technical reusability, recyclability (+0.25). Applies to producers, manufacturers, suppliers, importers (+0.25). Art. 20(2)(d) fine 15 min. wages for non-compliant placement.</t>
         </is>
       </c>
       <c r="V13" s="3">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>Annex I typology item 1.2: all plastic types including polystyrene foam. Packaging Standardisation System per IUCN.</t>
+          <t>Lexology Packaging Standardisation System. Annex I item 1.2: all plastic types including polystyrene foam.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I14" s="3" t="n">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Art. 18: Packaging normalisation symbols for reusable, recyclable or recoverable packaging must be adopted on packaging or labels — clearly visible, legible, and durable for packaging lifetime including after opening.</t>
+          <t>Art. 18: Mandatory symbols for reusable, recyclable or recoverable packaging on packaging or label — clearly visible, legible, lasting expected packaging lifetime (Lexology: Symbol and labelling of packaging).</t>
         </is>
       </c>
       <c r="S14" s="3" t="n">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="U14" s="2" t="inlineStr">
         <is>
-          <t>'devem ser adoptados símbolos específicos para as embalagens reutilizáveis, recicláveis ou valorizáveis' on packaging/labels. Information/labelling requirement (+0.25). Symbol standards not further specified in decree — implementation depends on complementary norms.</t>
+          <t>Lexology: 'use of specific symbols is mandatory' on packaging or label, visible and legible for packaging lifetime (+0.25). Symbol technical standards depend on complementary norms not yet specified.</t>
         </is>
       </c>
       <c r="V14" s="3">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="W14" s="2" t="inlineStr">
         <is>
-          <t>Information-type labelling; scored 0.40 per mandatory visibility requirement (Rule 10).</t>
+          <t>Lexology symbol/labelling requirement under Packaging Standardisation System.</t>
         </is>
       </c>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I15" s="3" t="n">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Art. 19: Environment Ministry fiscalizes Regulation compliance and decides on fines and accessory sanctions; Municipal Councils and District Administrations must collaborate by providing information for enforcement.</t>
+          <t>Art. 19: Environment Ministry supervises Regulation compliance; Municipal Councils and District Administrations cooperate in supervision (Lexology).</t>
         </is>
       </c>
       <c r="S15" s="3" t="n">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="U15" s="2" t="inlineStr">
         <is>
-          <t>'Compete ao Ministério que superintende a área do Ambiente fiscalizar o cumprimento do presente Regulamento.' Authority (+0.25), fine decision power linked to Arts. 20–22 (+0.25). Municipal collaboration duty (+0.25 monitoring).</t>
+          <t>Lexology: Environment Ministry 'responsible for the supervision' with municipal and district cooperation (+0.25 authority, +0.25 multi-level). Linked to Arts. 20–21 fine and ancillary sanction powers (+0.25).</t>
         </is>
       </c>
       <c r="V15" s="3">
@@ -1876,7 +1876,7 @@
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>Primary enforcement governance for EPR including plastic packaging.</t>
+          <t>Lexology supervision framework for EPR including plastic packaging.</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E16" s="2" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I16" s="3" t="n">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Art. 20–22: Administrative fines — obstruction of inspection (10 min. wages); refusal of used packaging/deposit refund, placing packaged products without waste management assurance, non-payment of TAE, or non-compliant packaging (15 min. wages each); 30% cumulative increase for repeat offences; accessory sanctions include seizure, activity suspension, compulsory removal; 20-day payment deadline.</t>
+          <t>Art. 20–21: Breaches sanctionable with fines of 10–15 times Minimum Salary; 30% increase on reoccurrence; ancillary sanctions per Art. 21 may be imposed together with fines (Lexology).</t>
         </is>
       </c>
       <c r="S16" s="3" t="n">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="U16" s="2" t="inlineStr">
         <is>
-          <t>'Constituem infracções... puníveis com sanção de multa correspondente a 10/15 Salários Mínimos.' Explicit fines (+0.25). TAE non-payment sanction (+0.25). Accessory sanctions Art. 21 (+0.25). Coercive fiscal execution via Juízo das Execuções Fiscais if unpaid (Art. 22).</t>
+          <t>Lexology: fines 'between 10 and 15 times the Minimum Salary', +30% reoccurrence; ancillary sanctions with fines (+0.25 each). Decreto Art. 20 specifies obstruction (10), TAE non-payment and packaging breaches (15). Coercive fiscal execution if unpaid (Art. 22).</t>
         </is>
       </c>
       <c r="V16" s="3">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>Economic enforcement; VdA flash confirms 10–15 minimum wage fine range.</t>
+          <t>Lexology economic enforcement. Companies liable for 'fines and ancillary sanctions in the event of breach' per Lexology observations.</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E17" s="2" t="n">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I17" s="3" t="n">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>Art. 23: Creates COMAGE (Comissão de Monitoria e Avaliação da Gestão de Embalagens) — multistakeholder consultative body to advise on packaging management, coordinate authorities and operators, monitor TAE revenue use, and propose legal improvements; operating costs funded by FNDS.</t>
+          <t>Art. 23: COMAGE (Comissão de Monitoria e Avaliação da Gestão de Embalagens / Commission for the Supervision and Evaluation of the Management of Packaging) — multistakeholder body; proper functioning required for Regulation effectiveness (Lexology observations).</t>
         </is>
       </c>
       <c r="S17" s="3" t="n">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="U17" s="2" t="inlineStr">
         <is>
-          <t>'É criada a Comissão de Monitoria e Avaliação da Gestão de Embalagens (COMAGE).' Body created (+0.25). Africa RISE/Imani 2022–2025 supported COMAGE operationalisation under MTA (+0.25). Consultative not executive — implementation depends on functioning secretariat and stakeholder participation.</t>
+          <t>Lexology: effectiveness 'will depend on... the proper functioning of' COMAGE (+0.25). Body created Art. 23 (+0.25). Africa RISE/Imani 2022–2025 supported operationalisation under MTA (+0.25). Consultative mandate limits executive enforcement power.</t>
         </is>
       </c>
       <c r="V17" s="3">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="W17" s="2" t="inlineStr">
         <is>
-          <t>Lexology/Africa RISE identify COMAGE as key EPR governance institution.</t>
+          <t>Lexology observations flag COMAGE as critical dependency for EPR effectiveness.</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E18" s="2" t="n">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I18" s="3" t="n">
@@ -2175,7 +2175,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Adopt principles, norms and guidelines assigning extended responsibility to producers and importers of packaging and packaging waste to protect public health and the environment within sustainable development, through internal management systems, the Packaging Environmental Fee (TAE), and packaging normalisation.</t>
+          <t>Adoption of principles, rules and guidelines to increase the responsibility of producers and importers of packaging in order to safeguard the environment and public health, in the context of sustainable development (Lexology; Reg. Art. 2).</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017 and published 28 December 2017 (Boletim da República), under Lei 20/97 Arts. 10 and 33. Sub-legislative EPR instrument, not parliamentary legislation.</t>
+          <t>Executive decree (Decreto n.º 79/2017) approved by the Council of Ministers on 21 November 2017, published 28 December 2017, entered into force 29 December 2017 (Lexology). Sub-legislative EPR instrument under Lei 20/97 Arts. 10 and 33.</t>
         </is>
       </c>
       <c r="I19" s="3" t="n">
@@ -2263,7 +2263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2329,7 +2329,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Analysis source (user)</t>
+          <t>Primary analysis</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2341,44 +2341,56 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Supplementary sources</t>
+          <t>Lexology text</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>VdA Legal Partners flash 2018; IUCN MARPLASTICCS 2022; Club of Mozambique/Lusa DM 26/2025; Imani Development Africa RISE 2022–2025</t>
+          <t>User-provided (incorporated in generator and Word doc)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Coding date</t>
+          <t>Implementation updates</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>June 2026</t>
+          <t>DM 26/2025 (March 2025); IUCN MARPLASTICCS 2022; Africa RISE/Imani Development 2022–2025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Total instrument rows</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>18</v>
+          <t>Coding date</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>June 2026</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Total instrument rows</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Columns O and V use Excel formulas. policy_score = AVERAGE(G,I,K,M,P); instrument_score = AVERAGE(P,T). TAE in_force updated to 1 following DM 26/2025 (March 2025).</t>
         </is>

</xml_diff>